<commit_message>
Lab 5: built-in visual skills only; Lab 6: custom Pareto-chart skill
- Lab 5 now focuses on @chart-design and @theme-design: four charts on a
  Charts sheet, a Checks sheet and one theme. The finance skills
  (@unit-economics, @check-model), the CAC/LTV content and the
  Headcount_Budget sheet are removed.
- Lab 6 replaces the interview-calendar skill with a pareto-chart skill:
  draft SKILL.md in Copilot on the web, save it, upload it to the OneDrive
  skills folder, install it in Excel and run it on a 500-row job-postings
  workbook (16 job categories, a different colour for every column).
- Deck, Lesson Plan, Learner Guide, prompts page and labs rebuilt from the
  single source; labs renamed to lab-05-built-in-skills-visual-design and
  lab-06-custom-skills-pareto-chart.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/labs/lab-01-data-prep-and-data-quality/data/BrightPath_Candidate_Pipeline.xlsx
+++ b/labs/lab-01-data-prep-and-data-quality/data/BrightPath_Candidate_Pipeline.xlsx
@@ -14235,7 +14235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14291,8 +14291,8 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Format the data on the Applications sheet (from A1 to the last row and column) as an Excel table with headers. Name the table tblApplications. Do not change, sort or delete any values.
-Then tell me the table name, the number of columns and the number of data rows.</t>
+          <t>Turn the data on the Applications sheet into a table named tblApplications. Don't change any values.
+Then tell me how many rows and columns it has.</t>
         </is>
       </c>
     </row>
@@ -14309,12 +14309,7 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>GOAL: Describe this candidate pipeline before I analyse it.
-CONTEXT: BrightPath recruitment desk, H1 2026. One row should be one application.
-DATA: Use only tblApplications.
-CONSTRAINTS: Do not change the workbook.
-OUTPUT: What a row represents, each column with its data type, the number of rows, the Applied_Date range and the distinct values of Stage and Source.
-REVIEW: Tell me how you counted the rows.</t>
+          <t>Describe this data for me. What does one row represent, what dates does it cover, and what are the different Stage and Source values?</t>
         </is>
       </c>
     </row>
@@ -14331,7 +14326,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Check tblApplications for data-quality issues. List any Application_ID that appears more than once, and any Source value that is not exactly one of: LinkedIn, JobStreet, MyCareersFuture, Referral, BrightPath Website, Job Fair, Talent Database. Give the count of each issue. Do not change anything.</t>
+          <t>Are there any data-quality problems in tblApplications, such as repeated Application_IDs or Source names spelt in different ways? Don't change anything yet.</t>
         </is>
       </c>
     </row>
@@ -14348,84 +14343,82 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>1) Highlight Application_ID cells that appear more than once in tblApplications with an orange fill.
-2) Add a column Source_Clean to tblApplications that trims spaces from Source and changes 'Linked In' to 'LinkedIn'. Do not delete or edit any existing values.</t>
+          <t>Highlight the repeated Application_IDs in orange. Then add a Source_Clean column with the Source names tidied up, and keep the original Source column as it is.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>4 · E</t>
+          <t>5 · E</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Plan</t>
+          <t>Chat only</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>For each duplicated Application_ID, give the row numbers of both copies and say whether the two rows are identical.</t>
+          <t>Which source brings in the most hires? Show the applications, hires and hire rate for each source, using Source_Clean.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>4 · F</t>
+          <t>5 · F</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Plan</t>
+          <t>Allow editing</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Highlight the Source cells in tblApplications where Source_Clean is different from Source with a yellow fill. Tell me how many cells you highlighted and list their Application_IDs.</t>
+          <t>Add a Checks sheet with formulas that count the total hires and the LinkedIn hires, so I can check your answer.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>4 · G</t>
+          <t>6 · G</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Plan</t>
+          <t>Allow editing</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>List the distinct Source_Clean values with a count of each. Confirm there is no 'Linked In' and no value with a trailing space, and that tblApplications still has 242 rows.</t>
+          <t>Highlight the rows of candidates who were hired in light green.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>5 · H</t>
+          <t>6 · H</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Chat only</t>
+          <t>Allow editing</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Using tblApplications, count applications and hires (Stage = "Hired") by Source_Clean.
-Show a table sorted by hires, highest first, with hire rate = hires / applications.</t>
+          <t>Sort the table so the highest interview scores come first.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>5 · I</t>
+          <t>6 · I</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -14435,299 +14428,109 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>On a sheet named Checks (create it if needed), add these formulas with a label beside each, then tell me the results:
-=COUNTIFS(tblApplications[Stage],"Hired")
-=COUNTIFS(tblApplications[Source_Clean],"LinkedIn",tblApplications[Stage],"Hired")</t>
+          <t>Show only the Technology candidates at the Interview stage. How many are there?</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>5 · J</t>
+          <t>7 · J</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Chat only</t>
+          <t>Allow editing</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Using tblApplications, count applications and hires (Stage = "Hired") by Source_Clean.
-Show a table sorted by hires, highest first.</t>
+          <t>Prompt_Log already lists every prompt in this lab. For each one I ran, fill in What Copilot did and How I verified, and set Decision to Keep. I will tell you any row to change to Revise or Undo.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>6 · K</t>
+          <t>Extra 1</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Allow editing</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Highlight entire rows of tblApplications where Stage is "Hired" with a light green fill.</t>
+          <t>Give me a quick summary of this pipeline data in five bullet points.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>6 · L</t>
+          <t>Extra 2</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Allow editing</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Sort tblApplications by Interview_Score from highest to lowest, then by Days_in_Pipeline from lowest to highest.</t>
+          <t>Which sector received the most applications?</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>6 · M</t>
+          <t>Extra 3</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Allow editing</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Filter tblApplications to show only Client_Sector = "Technology" and Stage = "Interview".</t>
+          <t>Which recruiter has the most candidates at the Offer stage?</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>6 · N</t>
+          <t>Extra 4</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Allow editing</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>How many rows of tblApplications are visible with this filter?</t>
+          <t>Highlight the candidates with an interview score of 5 in light blue.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>6 · O</t>
+          <t>Extra 5</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Allow editing</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Clear all filters on tblApplications and confirm all 242 rows are visible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>7 · P</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Allow editing</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>Prompt_Log already lists every prompt in this lab. For each one I ran, fill in What Copilot did and How I verified, and set Decision to Keep. I will tell you any row to change to Revise or Undo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>Extra 1</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>Describe tblApplications: what one row represents, each column's data type, the row count and the Applied_Date range. Do not change the workbook.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Extra 2</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>List any Application_ID that appears more than once in tblApplications and any Source value that is not in the canonical list on About_This_Data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Extra 3</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>Plan how you would flag duplicate Application_IDs and standardise Source. Show me the steps before you change anything.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Extra 4</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Add a column Source_Clean that trims spaces from Source and replaces 'Linked In' with 'LinkedIn'. Do not change the original Source column.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Extra 5</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>Using tblApplications, count applications and hires by Source_Clean and show the hire rate. Sort by hires, highest first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>Extra 6</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Which Client_Sector received the most applications, and how many? Show the count for every sector.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>Extra 7</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>Highlight rows where Stage is Hired in light green.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>Extra 8</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Sort tblApplications by Interview_Score from highest to lowest, then by Days_in_Pipeline from lowest to highest.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Extra 9</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Filter to show only Technology applications at the Interview stage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>Extra 10</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>What's interesting about this pipeline data? Give three observations, each with the numbers behind it.</t>
+          <t>What's interesting about this data? Give me three observations with the numbers behind them.</t>
         </is>
       </c>
     </row>

</xml_diff>